<commit_message>
Other vehicle data were updated
</commit_message>
<xml_diff>
--- a/pasto_case/results/AHP_results/matrix_criteria.xlsx
+++ b/pasto_case/results/AHP_results/matrix_criteria.xlsx
@@ -516,7 +516,7 @@
         <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>1.935</v>
+        <v>1.933</v>
       </c>
       <c r="E2" t="n">
         <v>1.035</v>
@@ -525,7 +525,7 @@
         <v>1.011</v>
       </c>
       <c r="G2" t="n">
-        <v>1.084</v>
+        <v>1.081</v>
       </c>
       <c r="H2" t="n">
         <v>1.074</v>
@@ -557,10 +557,10 @@
         <v>0.523</v>
       </c>
       <c r="G3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5590000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>0.555</v>
+        <v>0.556</v>
       </c>
       <c r="I3" t="n">
         <v>0.518</v>
@@ -580,7 +580,7 @@
         <v>0.966</v>
       </c>
       <c r="D4" t="n">
-        <v>1.87</v>
+        <v>1.868</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -589,7 +589,7 @@
         <v>0.977</v>
       </c>
       <c r="G4" t="n">
-        <v>1.048</v>
+        <v>1.045</v>
       </c>
       <c r="H4" t="n">
         <v>1.038</v>
@@ -612,7 +612,7 @@
         <v>0.989</v>
       </c>
       <c r="D5" t="n">
-        <v>1.913</v>
+        <v>1.912</v>
       </c>
       <c r="E5" t="n">
         <v>1.023</v>
@@ -621,7 +621,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>1.072</v>
+        <v>1.069</v>
       </c>
       <c r="H5" t="n">
         <v>1.062</v>
@@ -641,28 +641,28 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.922</v>
+        <v>0.925</v>
       </c>
       <c r="D6" t="n">
-        <v>1.785</v>
+        <v>1.788</v>
       </c>
       <c r="E6" t="n">
-        <v>0.954</v>
+        <v>0.957</v>
       </c>
       <c r="F6" t="n">
-        <v>0.9330000000000001</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>0.991</v>
+        <v>0.994</v>
       </c>
       <c r="I6" t="n">
-        <v>0.924</v>
+        <v>0.926</v>
       </c>
       <c r="J6" t="n">
-        <v>0.921</v>
+        <v>0.923</v>
       </c>
     </row>
     <row r="7">
@@ -676,7 +676,7 @@
         <v>0.931</v>
       </c>
       <c r="D7" t="n">
-        <v>1.801</v>
+        <v>1.8</v>
       </c>
       <c r="E7" t="n">
         <v>0.963</v>
@@ -685,7 +685,7 @@
         <v>0.9409999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>1.009</v>
+        <v>1.007</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -708,19 +708,19 @@
         <v>0.998</v>
       </c>
       <c r="D8" t="n">
-        <v>1.931</v>
+        <v>1.93</v>
       </c>
       <c r="E8" t="n">
         <v>1.033</v>
       </c>
       <c r="F8" t="n">
-        <v>1.009</v>
+        <v>1.01</v>
       </c>
       <c r="G8" t="n">
-        <v>1.082</v>
+        <v>1.079</v>
       </c>
       <c r="H8" t="n">
-        <v>1.073</v>
+        <v>1.072</v>
       </c>
       <c r="I8" t="n">
         <v>1</v>
@@ -740,7 +740,7 @@
         <v>1.002</v>
       </c>
       <c r="D9" t="n">
-        <v>1.938</v>
+        <v>1.937</v>
       </c>
       <c r="E9" t="n">
         <v>1.036</v>
@@ -749,7 +749,7 @@
         <v>1.013</v>
       </c>
       <c r="G9" t="n">
-        <v>1.086</v>
+        <v>1.083</v>
       </c>
       <c r="H9" t="n">
         <v>1.076</v>
@@ -776,25 +776,25 @@
         <v>1</v>
       </c>
       <c r="D10" t="n">
-        <v>1.075</v>
+        <v>1.078</v>
       </c>
       <c r="E10" t="n">
-        <v>1.075</v>
+        <v>1.078</v>
       </c>
       <c r="F10" t="n">
-        <v>1.075</v>
+        <v>1.078</v>
       </c>
       <c r="G10" t="n">
-        <v>1.2</v>
+        <v>1.168</v>
       </c>
       <c r="H10" t="n">
-        <v>1.021</v>
+        <v>1.022</v>
       </c>
       <c r="I10" t="n">
-        <v>1.021</v>
+        <v>1.022</v>
       </c>
       <c r="J10" t="n">
-        <v>1.021</v>
+        <v>1.022</v>
       </c>
     </row>
     <row r="11">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.93</v>
+        <v>0.928</v>
       </c>
       <c r="D11" t="n">
         <v>1</v>
@@ -817,16 +817,16 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>1.116</v>
+        <v>1.084</v>
       </c>
       <c r="H11" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="I11" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="J11" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
     </row>
     <row r="12">
@@ -837,7 +837,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.93</v>
+        <v>0.928</v>
       </c>
       <c r="D12" t="n">
         <v>1</v>
@@ -849,16 +849,16 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>1.116</v>
+        <v>1.084</v>
       </c>
       <c r="H12" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="I12" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="J12" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
     </row>
     <row r="13">
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.93</v>
+        <v>0.928</v>
       </c>
       <c r="D13" t="n">
         <v>1</v>
@@ -881,16 +881,16 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>1.116</v>
+        <v>1.084</v>
       </c>
       <c r="H13" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="I13" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
       <c r="J13" t="n">
-        <v>0.95</v>
+        <v>0.948</v>
       </c>
     </row>
     <row r="14">
@@ -901,28 +901,28 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.833</v>
+        <v>0.856</v>
       </c>
       <c r="D14" t="n">
-        <v>0.896</v>
+        <v>0.923</v>
       </c>
       <c r="E14" t="n">
-        <v>0.896</v>
+        <v>0.923</v>
       </c>
       <c r="F14" t="n">
-        <v>0.896</v>
+        <v>0.923</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>0.851</v>
+        <v>0.875</v>
       </c>
       <c r="I14" t="n">
-        <v>0.851</v>
+        <v>0.875</v>
       </c>
       <c r="J14" t="n">
-        <v>0.851</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="15">
@@ -933,19 +933,19 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.979</v>
+        <v>0.978</v>
       </c>
       <c r="D15" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="E15" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="F15" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="G15" t="n">
-        <v>1.175</v>
+        <v>1.143</v>
       </c>
       <c r="H15" t="n">
         <v>1</v>
@@ -965,19 +965,19 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.979</v>
+        <v>0.978</v>
       </c>
       <c r="D16" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="E16" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="F16" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="G16" t="n">
-        <v>1.175</v>
+        <v>1.143</v>
       </c>
       <c r="H16" t="n">
         <v>1</v>
@@ -997,19 +997,19 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.979</v>
+        <v>0.978</v>
       </c>
       <c r="D17" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="E17" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="F17" t="n">
-        <v>1.053</v>
+        <v>1.054</v>
       </c>
       <c r="G17" t="n">
-        <v>1.175</v>
+        <v>1.143</v>
       </c>
       <c r="H17" t="n">
         <v>1</v>
@@ -1036,25 +1036,25 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>0.48</v>
+        <v>0.39</v>
       </c>
       <c r="E18" t="n">
-        <v>0.48</v>
+        <v>0.39</v>
       </c>
       <c r="F18" t="n">
-        <v>0.492</v>
+        <v>0.407</v>
       </c>
       <c r="G18" t="n">
-        <v>0.146</v>
+        <v>0.157</v>
       </c>
       <c r="H18" t="n">
-        <v>0.785</v>
+        <v>0.765</v>
       </c>
       <c r="I18" t="n">
-        <v>0.785</v>
+        <v>0.765</v>
       </c>
       <c r="J18" t="n">
-        <v>0.786</v>
+        <v>0.765</v>
       </c>
     </row>
     <row r="19">
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.084</v>
+        <v>2.566</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -1074,19 +1074,19 @@
         <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>1.025</v>
+        <v>1.045</v>
       </c>
       <c r="G19" t="n">
-        <v>0.305</v>
+        <v>0.402</v>
       </c>
       <c r="H19" t="n">
-        <v>1.636</v>
+        <v>1.963</v>
       </c>
       <c r="I19" t="n">
-        <v>1.636</v>
+        <v>1.963</v>
       </c>
       <c r="J19" t="n">
-        <v>1.637</v>
+        <v>1.964</v>
       </c>
     </row>
     <row r="20">
@@ -1097,7 +1097,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2.084</v>
+        <v>2.566</v>
       </c>
       <c r="D20" t="n">
         <v>1</v>
@@ -1106,19 +1106,19 @@
         <v>1</v>
       </c>
       <c r="F20" t="n">
-        <v>1.025</v>
+        <v>1.045</v>
       </c>
       <c r="G20" t="n">
-        <v>0.305</v>
+        <v>0.402</v>
       </c>
       <c r="H20" t="n">
-        <v>1.636</v>
+        <v>1.963</v>
       </c>
       <c r="I20" t="n">
-        <v>1.636</v>
+        <v>1.963</v>
       </c>
       <c r="J20" t="n">
-        <v>1.637</v>
+        <v>1.964</v>
       </c>
     </row>
     <row r="21">
@@ -1129,28 +1129,28 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2.033</v>
+        <v>2.456</v>
       </c>
       <c r="D21" t="n">
-        <v>0.975</v>
+        <v>0.957</v>
       </c>
       <c r="E21" t="n">
-        <v>0.975</v>
+        <v>0.957</v>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>0.297</v>
+        <v>0.385</v>
       </c>
       <c r="H21" t="n">
-        <v>1.596</v>
+        <v>1.879</v>
       </c>
       <c r="I21" t="n">
-        <v>1.596</v>
+        <v>1.879</v>
       </c>
       <c r="J21" t="n">
-        <v>1.597</v>
+        <v>1.88</v>
       </c>
     </row>
     <row r="22">
@@ -1161,28 +1161,28 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6.836</v>
+        <v>6.388</v>
       </c>
       <c r="D22" t="n">
-        <v>3.28</v>
+        <v>2.489</v>
       </c>
       <c r="E22" t="n">
-        <v>3.28</v>
+        <v>2.489</v>
       </c>
       <c r="F22" t="n">
-        <v>3.363</v>
+        <v>2.6</v>
       </c>
       <c r="G22" t="n">
         <v>1</v>
       </c>
       <c r="H22" t="n">
-        <v>5.368</v>
+        <v>4.887</v>
       </c>
       <c r="I22" t="n">
-        <v>5.368</v>
+        <v>4.887</v>
       </c>
       <c r="J22" t="n">
-        <v>5.37</v>
+        <v>4.889</v>
       </c>
     </row>
     <row r="23">
@@ -1193,19 +1193,19 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.273</v>
+        <v>1.307</v>
       </c>
       <c r="D23" t="n">
-        <v>0.611</v>
+        <v>0.509</v>
       </c>
       <c r="E23" t="n">
-        <v>0.611</v>
+        <v>0.509</v>
       </c>
       <c r="F23" t="n">
-        <v>0.626</v>
+        <v>0.532</v>
       </c>
       <c r="G23" t="n">
-        <v>0.186</v>
+        <v>0.205</v>
       </c>
       <c r="H23" t="n">
         <v>1</v>
@@ -1225,19 +1225,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1.273</v>
+        <v>1.307</v>
       </c>
       <c r="D24" t="n">
-        <v>0.611</v>
+        <v>0.509</v>
       </c>
       <c r="E24" t="n">
-        <v>0.611</v>
+        <v>0.509</v>
       </c>
       <c r="F24" t="n">
-        <v>0.626</v>
+        <v>0.532</v>
       </c>
       <c r="G24" t="n">
-        <v>0.186</v>
+        <v>0.205</v>
       </c>
       <c r="H24" t="n">
         <v>1</v>
@@ -1257,19 +1257,19 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1.273</v>
+        <v>1.306</v>
       </c>
       <c r="D25" t="n">
-        <v>0.611</v>
+        <v>0.509</v>
       </c>
       <c r="E25" t="n">
-        <v>0.611</v>
+        <v>0.509</v>
       </c>
       <c r="F25" t="n">
-        <v>0.626</v>
+        <v>0.532</v>
       </c>
       <c r="G25" t="n">
-        <v>0.186</v>
+        <v>0.205</v>
       </c>
       <c r="H25" t="n">
         <v>1</v>
@@ -1305,16 +1305,16 @@
         <v>0.111</v>
       </c>
       <c r="G26" t="n">
-        <v>0.333</v>
+        <v>0.2</v>
       </c>
       <c r="H26" t="n">
-        <v>0.167</v>
+        <v>0.143</v>
       </c>
       <c r="I26" t="n">
-        <v>0.167</v>
+        <v>0.143</v>
       </c>
       <c r="J26" t="n">
-        <v>0.167</v>
+        <v>0.143</v>
       </c>
     </row>
     <row r="27">
@@ -1337,16 +1337,16 @@
         <v>1</v>
       </c>
       <c r="G27" t="n">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="H27" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
       <c r="I27" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
       <c r="J27" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
     </row>
     <row r="28">
@@ -1369,16 +1369,16 @@
         <v>1</v>
       </c>
       <c r="G28" t="n">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="H28" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
       <c r="I28" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
       <c r="J28" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
     </row>
     <row r="29">
@@ -1401,16 +1401,16 @@
         <v>1</v>
       </c>
       <c r="G29" t="n">
-        <v>3</v>
+        <v>1.8</v>
       </c>
       <c r="H29" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
       <c r="I29" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
       <c r="J29" t="n">
-        <v>1.5</v>
+        <v>1.286</v>
       </c>
     </row>
     <row r="30">
@@ -1421,28 +1421,28 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>0.333</v>
+        <v>0.556</v>
       </c>
       <c r="E30" t="n">
-        <v>0.333</v>
+        <v>0.556</v>
       </c>
       <c r="F30" t="n">
-        <v>0.333</v>
+        <v>0.556</v>
       </c>
       <c r="G30" t="n">
         <v>1</v>
       </c>
       <c r="H30" t="n">
-        <v>0.5</v>
+        <v>0.714</v>
       </c>
       <c r="I30" t="n">
-        <v>0.5</v>
+        <v>0.714</v>
       </c>
       <c r="J30" t="n">
-        <v>0.5</v>
+        <v>0.714</v>
       </c>
     </row>
     <row r="31">
@@ -1453,19 +1453,19 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D31" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="E31" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="F31" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="G31" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="H31" t="n">
         <v>1</v>
@@ -1485,19 +1485,19 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D32" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="E32" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="F32" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="G32" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="H32" t="n">
         <v>1</v>
@@ -1517,19 +1517,19 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D33" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="E33" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="F33" t="n">
-        <v>0.667</v>
+        <v>0.778</v>
       </c>
       <c r="G33" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="H33" t="n">
         <v>1</v>
@@ -1556,25 +1556,25 @@
         <v>1</v>
       </c>
       <c r="D34" t="n">
-        <v>0.165</v>
+        <v>0.001</v>
       </c>
       <c r="E34" t="n">
-        <v>0.165</v>
+        <v>0.001</v>
       </c>
       <c r="F34" t="n">
-        <v>0.165</v>
+        <v>0.001</v>
       </c>
       <c r="G34" t="n">
-        <v>0.669</v>
+        <v>0.772</v>
       </c>
       <c r="H34" t="n">
-        <v>0.133</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>0.133</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>0.133</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -1585,7 +1585,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>6.054</v>
+        <v>1604.337</v>
       </c>
       <c r="D35" t="n">
         <v>1</v>
@@ -1597,16 +1597,16 @@
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>4.048</v>
+        <v>1239.339</v>
       </c>
       <c r="H35" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
       <c r="I35" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
       <c r="J35" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
     </row>
     <row r="36">
@@ -1617,7 +1617,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>6.054</v>
+        <v>1604.337</v>
       </c>
       <c r="D36" t="n">
         <v>1</v>
@@ -1629,16 +1629,16 @@
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>4.048</v>
+        <v>1239.339</v>
       </c>
       <c r="H36" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
       <c r="I36" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
       <c r="J36" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
     </row>
     <row r="37">
@@ -1649,7 +1649,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6.054</v>
+        <v>1604.337</v>
       </c>
       <c r="D37" t="n">
         <v>1</v>
@@ -1661,16 +1661,16 @@
         <v>1</v>
       </c>
       <c r="G37" t="n">
-        <v>4.048</v>
+        <v>1239.339</v>
       </c>
       <c r="H37" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
       <c r="I37" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
       <c r="J37" t="n">
-        <v>0.806</v>
+        <v>0.648</v>
       </c>
     </row>
     <row r="38">
@@ -1681,28 +1681,28 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1.496</v>
+        <v>1.295</v>
       </c>
       <c r="D38" t="n">
-        <v>0.247</v>
+        <v>0.001</v>
       </c>
       <c r="E38" t="n">
-        <v>0.247</v>
+        <v>0.001</v>
       </c>
       <c r="F38" t="n">
-        <v>0.247</v>
+        <v>0.001</v>
       </c>
       <c r="G38" t="n">
         <v>1</v>
       </c>
       <c r="H38" t="n">
-        <v>0.199</v>
+        <v>0.001</v>
       </c>
       <c r="I38" t="n">
-        <v>0.199</v>
+        <v>0.001</v>
       </c>
       <c r="J38" t="n">
-        <v>0.199</v>
+        <v>0.001</v>
       </c>
     </row>
     <row r="39">
@@ -1713,19 +1713,19 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>7.514</v>
+        <v>2477.493</v>
       </c>
       <c r="D39" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="E39" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="F39" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="G39" t="n">
-        <v>5.023</v>
+        <v>1913.845</v>
       </c>
       <c r="H39" t="n">
         <v>1</v>
@@ -1745,19 +1745,19 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7.514</v>
+        <v>2477.493</v>
       </c>
       <c r="D40" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="E40" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="F40" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="G40" t="n">
-        <v>5.023</v>
+        <v>1913.845</v>
       </c>
       <c r="H40" t="n">
         <v>1</v>
@@ -1777,19 +1777,19 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>7.514</v>
+        <v>2477.493</v>
       </c>
       <c r="D41" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="E41" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="F41" t="n">
-        <v>1.241</v>
+        <v>1.544</v>
       </c>
       <c r="G41" t="n">
-        <v>5.023</v>
+        <v>1913.845</v>
       </c>
       <c r="H41" t="n">
         <v>1</v>

</xml_diff>